<commit_message>
Prepare mortgage forbearance case study for publication
</commit_message>
<xml_diff>
--- a/testing/mortgage-forbearance-test-scenarios.xlsx
+++ b/testing/mortgage-forbearance-test-scenarios.xlsx
@@ -5,15 +5,20 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t_all\Documents\Business Analyst 30 days Preparation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t_all\Documents\Portfolio\mortgage-forbearance-control-analysis\testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0230FA6E-C865-49D2-ACB2-35880595CCAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84AECDD6-633D-486C-885D-83883D6B6CC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-1260" windowWidth="29040" windowHeight="15720" xr2:uid="{9B47F4EF-8FFA-4FFC-812A-059F7CEAD3B1}"/>
+    <workbookView xWindow="-28920" yWindow="-1260" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="5" xr2:uid="{9B47F4EF-8FFA-4FFC-812A-059F7CEAD3B1}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
+    <sheet name="Traceability Matrix" sheetId="2" r:id="rId2"/>
+    <sheet name="Requirements Register" sheetId="3" r:id="rId3"/>
+    <sheet name="Business Rules Register" sheetId="4" r:id="rId4"/>
+    <sheet name="Exception Rules Register" sheetId="5" r:id="rId5"/>
+    <sheet name="Non-Functional Requirements" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="382">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -98,9 +103,6 @@
     <t>TC-002</t>
   </si>
   <si>
-    <t>TL-FR-003, -RULE-001</t>
-  </si>
-  <si>
     <t>Create a controlled mortgage-forbearance case with all mandatory information</t>
   </si>
   <si>
@@ -258,6 +260,936 @@
   </si>
   <si>
     <t>The reviewer can see the material actions, timestamps, users or systems involved, policy version, rule results, rationale, approval details, approved version and execution result in chronological order.</t>
+  </si>
+  <si>
+    <t>TL-FR-003, TL-RULE-001</t>
+  </si>
+  <si>
+    <t>Requirement Description</t>
+  </si>
+  <si>
+    <t>Jira Story</t>
+  </si>
+  <si>
+    <t>Acceptance Criteria</t>
+  </si>
+  <si>
+    <t>Coverage Status</t>
+  </si>
+  <si>
+    <t>Requirement Type</t>
+  </si>
+  <si>
+    <t>Source / Rationale</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Related Process Step</t>
+  </si>
+  <si>
+    <t>Related Rule ID</t>
+  </si>
+  <si>
+    <t>Rule ID</t>
+  </si>
+  <si>
+    <t>Rule Description</t>
+  </si>
+  <si>
+    <t>Rule Type</t>
+  </si>
+  <si>
+    <t>Trigger / Condition</t>
+  </si>
+  <si>
+    <t>Expected Behaviour</t>
+  </si>
+  <si>
+    <t>Related Requirement ID</t>
+  </si>
+  <si>
+    <t>TL-FR-001</t>
+  </si>
+  <si>
+    <t>Functional</t>
+  </si>
+  <si>
+    <t>The proposed solution shall allow an authorised operator to create a mortgage-forbearance case.</t>
+  </si>
+  <si>
+    <t>Supports controlled intake from the start of the process.</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Draft</t>
+  </si>
+  <si>
+    <t>Case creation</t>
+  </si>
+  <si>
+    <t>TL-FR-002</t>
+  </si>
+  <si>
+    <t>The proposed solution shall capture mandatory customer, account and case information.</t>
+  </si>
+  <si>
+    <t>Supports complete assessment evidence.</t>
+  </si>
+  <si>
+    <t>TL-RULE-001</t>
+  </si>
+  <si>
+    <t>TL-FR-003</t>
+  </si>
+  <si>
+    <t>The proposed solution shall identify missing mandatory information before the case progresses to assessment.</t>
+  </si>
+  <si>
+    <t>Supports evidence-validation control.</t>
+  </si>
+  <si>
+    <t>Evidence validation</t>
+  </si>
+  <si>
+    <t>TL-FR-004</t>
+  </si>
+  <si>
+    <t>The proposed solution shall evaluate the case against the applicable policy criteria.</t>
+  </si>
+  <si>
+    <t>Supports policy evaluation.</t>
+  </si>
+  <si>
+    <t>Policy evaluation</t>
+  </si>
+  <si>
+    <t>TL-RULE-002</t>
+  </si>
+  <si>
+    <t>TL-FR-005</t>
+  </si>
+  <si>
+    <t>The proposed solution shall record the policy version used during assessment.</t>
+  </si>
+  <si>
+    <t>Supports later reconstruction of the decision.</t>
+  </si>
+  <si>
+    <t>TL-FR-006</t>
+  </si>
+  <si>
+    <t>The proposed solution shall record the proposed outcome and supporting rationale.</t>
+  </si>
+  <si>
+    <t>Links the assessment to the recommended decision.</t>
+  </si>
+  <si>
+    <t>Assessment outcome</t>
+  </si>
+  <si>
+    <t>TL-RULE-003</t>
+  </si>
+  <si>
+    <t>TL-FR-007</t>
+  </si>
+  <si>
+    <t>The proposed solution shall route cases requiring approval to an authorised approver.</t>
+  </si>
+  <si>
+    <t>Supports independent approval.</t>
+  </si>
+  <si>
+    <t>Approval</t>
+  </si>
+  <si>
+    <t>TL-RULE-004</t>
+  </si>
+  <si>
+    <t>TL-FR-008</t>
+  </si>
+  <si>
+    <t>The proposed solution shall prevent the case originator from approving their own case where segregation of duties applies.</t>
+  </si>
+  <si>
+    <t>Supports separation of duties.</t>
+  </si>
+  <si>
+    <t>TL-RULE-005</t>
+  </si>
+  <si>
+    <t>TL-FR-009</t>
+  </si>
+  <si>
+    <t>The proposed solution shall allow an authorised approver to approve, reject or return a case for further information.</t>
+  </si>
+  <si>
+    <t>Supports controlled approval outcomes.</t>
+  </si>
+  <si>
+    <t>TL-FR-010</t>
+  </si>
+  <si>
+    <t>The proposed solution shall record the final approved decision and its decision version.</t>
+  </si>
+  <si>
+    <t>Supports version-controlled approval evidence.</t>
+  </si>
+  <si>
+    <t>TL-RULE-006</t>
+  </si>
+  <si>
+    <t>TL-FR-011</t>
+  </si>
+  <si>
+    <t>The proposed solution shall prevent execution where the requested decision version does not match the approved decision version.</t>
+  </si>
+  <si>
+    <t>Central exact-match execution control.</t>
+  </si>
+  <si>
+    <t>Highest</t>
+  </si>
+  <si>
+    <t>Execution validation</t>
+  </si>
+  <si>
+    <t>Central control question in README</t>
+  </si>
+  <si>
+    <t>TL-FR-012</t>
+  </si>
+  <si>
+    <t>The proposed solution shall record the execution result and execution reference.</t>
+  </si>
+  <si>
+    <t>Supports comparison between approved and implemented outcome.</t>
+  </si>
+  <si>
+    <t>Execution result</t>
+  </si>
+  <si>
+    <t>TL-RULE-009</t>
+  </si>
+  <si>
+    <t>TL-FR-013</t>
+  </si>
+  <si>
+    <t>The proposed solution shall retain a history of material case actions and status changes.</t>
+  </si>
+  <si>
+    <t>Supports traceability and later review.</t>
+  </si>
+  <si>
+    <t>Audit history</t>
+  </si>
+  <si>
+    <t>TL-RULE-010</t>
+  </si>
+  <si>
+    <t>TL-FR-014</t>
+  </si>
+  <si>
+    <t>The proposed solution shall allow authorised reviewers to reconstruct the decision history of a case.</t>
+  </si>
+  <si>
+    <t>Supports audit, compliance and QA review.</t>
+  </si>
+  <si>
+    <t>Exception Handling</t>
+  </si>
+  <si>
+    <t>A case must not progress to assessment while mandatory evidence is incomplete.</t>
+  </si>
+  <si>
+    <t>Validation rule</t>
+  </si>
+  <si>
+    <t>Required evidence is missing</t>
+  </si>
+  <si>
+    <t>Block progression and identify missing information</t>
+  </si>
+  <si>
+    <t>Case may proceed only where an explicitly authorised exception applies</t>
+  </si>
+  <si>
+    <t>TL-FR-002, TL-FR-003</t>
+  </si>
+  <si>
+    <t>The policy version and applicable policy checks must be associated with the assessment.</t>
+  </si>
+  <si>
+    <t>Policy rule</t>
+  </si>
+  <si>
+    <t>Case is evaluated</t>
+  </si>
+  <si>
+    <t>Record policy version and rule results</t>
+  </si>
+  <si>
+    <t>Failed rules follow the controlled exception path</t>
+  </si>
+  <si>
+    <t>TL-FR-004, TL-FR-005</t>
+  </si>
+  <si>
+    <t>Each proposed decision must include a recorded rationale.</t>
+  </si>
+  <si>
+    <t>Decision rule</t>
+  </si>
+  <si>
+    <t>Proposed outcome is created</t>
+  </si>
+  <si>
+    <t>Require rationale before submission</t>
+  </si>
+  <si>
+    <t>Incomplete rationale blocks submission</t>
+  </si>
+  <si>
+    <t>Cases requiring approval must be routed to an authorised approver.</t>
+  </si>
+  <si>
+    <t>Approval rule</t>
+  </si>
+  <si>
+    <t>Assessment requires approval</t>
+  </si>
+  <si>
+    <t>Route to an authorised approval role</t>
+  </si>
+  <si>
+    <t>Unauthorised approval attempt is blocked</t>
+  </si>
+  <si>
+    <t>TL-FR-007, TL-FR-009</t>
+  </si>
+  <si>
+    <t>A case originator must not approve their own case where segregation of duties applies.</t>
+  </si>
+  <si>
+    <t>Segregation-of-duties rule</t>
+  </si>
+  <si>
+    <t>Originator attempts approval</t>
+  </si>
+  <si>
+    <t>Block approval</t>
+  </si>
+  <si>
+    <t>Case remains pending for an independent approver</t>
+  </si>
+  <si>
+    <t>The decision version submitted for execution must match the exact approved decision version.</t>
+  </si>
+  <si>
+    <t>Execution control</t>
+  </si>
+  <si>
+    <t>Execution is requested</t>
+  </si>
+  <si>
+    <t>Compare requested and approved versions; allow only exact match</t>
+  </si>
+  <si>
+    <t>Block execution and record mismatch</t>
+  </si>
+  <si>
+    <t>TL-FR-010, TL-FR-011</t>
+  </si>
+  <si>
+    <t>Central project control</t>
+  </si>
+  <si>
+    <t>TL-RULE-007</t>
+  </si>
+  <si>
+    <t>A material case change after approval invalidates or supersedes the previous approval.</t>
+  </si>
+  <si>
+    <t>Version-control rule</t>
+  </si>
+  <si>
+    <t>Material case information changes after approval</t>
+  </si>
+  <si>
+    <t>Require reassessment and new approval</t>
+  </si>
+  <si>
+    <t>Previous approval must not be used for execution</t>
+  </si>
+  <si>
+    <t>TL-RULE-008</t>
+  </si>
+  <si>
+    <t>An approved decision must not be altered without creating a new controlled version.</t>
+  </si>
+  <si>
+    <t>Approved decision is changed</t>
+  </si>
+  <si>
+    <t>Create a new decision version</t>
+  </si>
+  <si>
+    <t>Previous version remains part of the audit history</t>
+  </si>
+  <si>
+    <t>The execution result must remain linked to the approved decision record.</t>
+  </si>
+  <si>
+    <t>Execution-result rule</t>
+  </si>
+  <si>
+    <t>Execution completes or fails</t>
+  </si>
+  <si>
+    <t>Record result, status and reference against the approved decision</t>
+  </si>
+  <si>
+    <t>Failed execution remains incomplete and is investigated</t>
+  </si>
+  <si>
+    <t>Material case actions must record who or what performed the action and when.</t>
+  </si>
+  <si>
+    <t>Audit rule</t>
+  </si>
+  <si>
+    <t>Material action or status change occurs</t>
+  </si>
+  <si>
+    <t>Record actor, action and timestamp</t>
+  </si>
+  <si>
+    <t>Missing audit evidence should be treated as a control issue</t>
+  </si>
+  <si>
+    <t>TL-FR-013, TL-FR-014</t>
+  </si>
+  <si>
+    <t>Allow an authorised operator to create a mortgage-forbearance case.</t>
+  </si>
+  <si>
+    <t>SCRUM-1 – Capture a controlled mortgage-forbearance case</t>
+  </si>
+  <si>
+    <t>Authorised operator can create a case; unique ID and Draft status recorded.</t>
+  </si>
+  <si>
+    <t>Mapped</t>
+  </si>
+  <si>
+    <t>Positive-path test designed</t>
+  </si>
+  <si>
+    <t>Capture mandatory customer, account and case information.</t>
+  </si>
+  <si>
+    <t>Mandatory customer, account and case information can be recorded.</t>
+  </si>
+  <si>
+    <t>Identify missing mandatory information before assessment.</t>
+  </si>
+  <si>
+    <t>SCRUM-2 – Validate mandatory case information</t>
+  </si>
+  <si>
+    <t>Missing mandatory information is identified and blocks progression.</t>
+  </si>
+  <si>
+    <t>Negative-path test designed</t>
+  </si>
+  <si>
+    <t>Evaluate the case against applicable policy criteria.</t>
+  </si>
+  <si>
+    <t>SCRUM-3 – Evaluate the case against policy criteria</t>
+  </si>
+  <si>
+    <t>Applicable policy rules are evaluated and results recorded.</t>
+  </si>
+  <si>
+    <t>Partial</t>
+  </si>
+  <si>
+    <t>Exception path tested; add positive policy-evaluation scenario later</t>
+  </si>
+  <si>
+    <t>Record the policy version used during assessment.</t>
+  </si>
+  <si>
+    <t>Policy version is recorded against the case.</t>
+  </si>
+  <si>
+    <t>Audit scenario checks visibility; direct recording test not yet defined</t>
+  </si>
+  <si>
+    <t>Record proposed outcome and supporting rationale.</t>
+  </si>
+  <si>
+    <t>Proposed outcome and rationale must be recorded before completion.</t>
+  </si>
+  <si>
+    <t>Gap</t>
+  </si>
+  <si>
+    <t>No direct test scenario currently defined</t>
+  </si>
+  <si>
+    <t>Route cases requiring approval to an authorised approver.</t>
+  </si>
+  <si>
+    <t>SCRUM-4 – Submit the proposed outcome for independent approval</t>
+  </si>
+  <si>
+    <t>Case routes only to a user with required approval authority.</t>
+  </si>
+  <si>
+    <t>TC-003, TC-007</t>
+  </si>
+  <si>
+    <t>Tests approval controls but not routing directly</t>
+  </si>
+  <si>
+    <t>Prevent self-approval where segregation of duties applies.</t>
+  </si>
+  <si>
+    <t>SCRUM-4 / SCRUM-5</t>
+  </si>
+  <si>
+    <t>Case originator cannot approve their own case.</t>
+  </si>
+  <si>
+    <t>Direct negative-control test</t>
+  </si>
+  <si>
+    <t>Allow authorised approver to approve, reject or return a case.</t>
+  </si>
+  <si>
+    <t>SCRUM-5 – Review and decide a submitted case</t>
+  </si>
+  <si>
+    <t>Approver can approve, reject or return with required comments.</t>
+  </si>
+  <si>
+    <t>Direct approval-outcome test still required</t>
+  </si>
+  <si>
+    <t>Record final approved decision and decision version.</t>
+  </si>
+  <si>
+    <t>SCRUM-5 / SCRUM-6</t>
+  </si>
+  <si>
+    <t>Approval records approver, timestamp and approved version.</t>
+  </si>
+  <si>
+    <t>TC-004, TC-005, TC-006</t>
+  </si>
+  <si>
+    <t>Version-dependent tests designed</t>
+  </si>
+  <si>
+    <t>Prevent execution where requested version differs from approved version.</t>
+  </si>
+  <si>
+    <t>SCRUM-6 – Execute only the approved decision version</t>
+  </si>
+  <si>
+    <t>Execution allowed only where requested and approved versions match.</t>
+  </si>
+  <si>
+    <t>Core exact-match control covered</t>
+  </si>
+  <si>
+    <t>Record execution result and reference.</t>
+  </si>
+  <si>
+    <t>Successful or failed execution result is recorded.</t>
+  </si>
+  <si>
+    <t>TC-005, TC-009</t>
+  </si>
+  <si>
+    <t>Both success and failure paths covered</t>
+  </si>
+  <si>
+    <t>Retain history of material case actions and status changes.</t>
+  </si>
+  <si>
+    <t>SCRUM-8 – Reconstruct the complete decision history</t>
+  </si>
+  <si>
+    <t>Material actions include actor/system, timestamp and action.</t>
+  </si>
+  <si>
+    <t>Audit-history test designed</t>
+  </si>
+  <si>
+    <t>Allow authorised reviewers to reconstruct decision history.</t>
+  </si>
+  <si>
+    <t>Reviewer can see evidence, rules, rationale, approval and execution history.</t>
+  </si>
+  <si>
+    <t>Direct reconstruction scenario</t>
+  </si>
+  <si>
+    <t>Case cannot progress while mandatory evidence is incomplete.</t>
+  </si>
+  <si>
+    <t>SCRUM-2</t>
+  </si>
+  <si>
+    <t>Missing mandatory information blocks progression unless authorised exception applies.</t>
+  </si>
+  <si>
+    <t>Direct negative-path test</t>
+  </si>
+  <si>
+    <t>Policy version and applicable rule results must be associated with the assessment.</t>
+  </si>
+  <si>
+    <t>SCRUM-3</t>
+  </si>
+  <si>
+    <t>Policy version and individual rule results are recorded.</t>
+  </si>
+  <si>
+    <t>TC-007, TC-010</t>
+  </si>
+  <si>
+    <t>Direct positive test still desirable</t>
+  </si>
+  <si>
+    <t>Every proposed decision must contain a recorded rationale.</t>
+  </si>
+  <si>
+    <t>SCRUM-3 / SCRUM-4</t>
+  </si>
+  <si>
+    <t>Submission blocked if rationale is absent.</t>
+  </si>
+  <si>
+    <t>Add negative rationale test</t>
+  </si>
+  <si>
+    <t>Cases requiring approval must go to an authorised approver.</t>
+  </si>
+  <si>
+    <t>Unauthorised approval is prevented.</t>
+  </si>
+  <si>
+    <t>Direct routing/authority test still desirable</t>
+  </si>
+  <si>
+    <t>Originator cannot approve own case where segregation of duties applies.</t>
+  </si>
+  <si>
+    <t>Self-approval is blocked.</t>
+  </si>
+  <si>
+    <t>Direct control test</t>
+  </si>
+  <si>
+    <t>Execution version must exactly match the approved decision version.</t>
+  </si>
+  <si>
+    <t>SCRUM-6</t>
+  </si>
+  <si>
+    <t>Exact match permits execution; mismatch blocks execution.</t>
+  </si>
+  <si>
+    <t>TC-004, TC-005</t>
+  </si>
+  <si>
+    <t>Material change after approval invalidates or supersedes previous approval.</t>
+  </si>
+  <si>
+    <t>SCRUM-4 / SCRUM-6</t>
+  </si>
+  <si>
+    <t>Material change requires reassessment and new approval.</t>
+  </si>
+  <si>
+    <t>Direct stale-approval test</t>
+  </si>
+  <si>
+    <t>Approved decision cannot be altered without creating a new controlled version.</t>
+  </si>
+  <si>
+    <t>Changed approved decision creates a new controlled version.</t>
+  </si>
+  <si>
+    <t>No direct version-creation test yet</t>
+  </si>
+  <si>
+    <t>Execution result must remain linked to the approved decision.</t>
+  </si>
+  <si>
+    <t>SCRUM-6 / SCRUM-8</t>
+  </si>
+  <si>
+    <t>Execution outcome and reference remain associated with approved decision.</t>
+  </si>
+  <si>
+    <t>Success and failure paths designed</t>
+  </si>
+  <si>
+    <t>Material actions must record actor/system and timestamp.</t>
+  </si>
+  <si>
+    <t>SCRUM-8</t>
+  </si>
+  <si>
+    <t>Full chronological history identifies who/what acted and when.</t>
+  </si>
+  <si>
+    <t>Audit scenario designed</t>
+  </si>
+  <si>
+    <t>Exception ID</t>
+  </si>
+  <si>
+    <t>Exception Rule</t>
+  </si>
+  <si>
+    <t>Required Approval / Control</t>
+  </si>
+  <si>
+    <t>Related Requirement / Rule</t>
+  </si>
+  <si>
+    <t>TL-EX-002</t>
+  </si>
+  <si>
+    <t>A policy exception must include a recorded reason, supporting evidence and authorised approval.</t>
+  </si>
+  <si>
+    <t>A case fails a policy rule but an exception is being requested.</t>
+  </si>
+  <si>
+    <t>Record the exception reason and evidence, then route the case for authorised review before progression.</t>
+  </si>
+  <si>
+    <t>Approval by a user with the required authority.</t>
+  </si>
+  <si>
+    <t>TL-RULE-004, TL-FR-007</t>
+  </si>
+  <si>
+    <t>Supports controlled policy-exception handling.</t>
+  </si>
+  <si>
+    <t>TL-EX-004</t>
+  </si>
+  <si>
+    <t>A material case change after approval must invalidate or supersede the previous approval.</t>
+  </si>
+  <si>
+    <t>Material case information changes after approval.</t>
+  </si>
+  <si>
+    <t>Prevent use of the previous approval and require reassessment and new approval.</t>
+  </si>
+  <si>
+    <t>New approval required before execution.</t>
+  </si>
+  <si>
+    <t>TL-RULE-007, TL-FR-010, TL-FR-011</t>
+  </si>
+  <si>
+    <t>Supports stale-approval control.</t>
+  </si>
+  <si>
+    <t>TL-EX-005</t>
+  </si>
+  <si>
+    <t>A failed execution must not be treated as a successfully completed customer outcome.</t>
+  </si>
+  <si>
+    <t>Mortgage servicing returns an execution failure.</t>
+  </si>
+  <si>
+    <t>Record the failure, keep the case incomplete and route the failure for investigation or further action.</t>
+  </si>
+  <si>
+    <t>Execution result must be recorded and reviewed.</t>
+  </si>
+  <si>
+    <t>TL-RULE-009, TL-FR-012</t>
+  </si>
+  <si>
+    <t>Supports execution-failure handling.</t>
+  </si>
+  <si>
+    <t>An execution authorisation that has expired or already been used must not permit another execution.</t>
+  </si>
+  <si>
+    <t>Execution is attempted using an invalid or previously consumed authorisation.</t>
+  </si>
+  <si>
+    <t>Block execution and record the attempted reuse or expiry.</t>
+  </si>
+  <si>
+    <t>Authorisation validity must be checked before execution.</t>
+  </si>
+  <si>
+    <t>Supports duplicate-execution prevention.</t>
+  </si>
+  <si>
+    <t>NFR ID</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Rationale</t>
+  </si>
+  <si>
+    <t>Related Process / Control</t>
+  </si>
+  <si>
+    <t>TL-NFR-005</t>
+  </si>
+  <si>
+    <t>Auditability</t>
+  </si>
+  <si>
+    <t>Material actions must be timestamped and attributable to a specific user or system.</t>
+  </si>
+  <si>
+    <t>Supports reconstruction of who or what performed each controlled action and when.</t>
+  </si>
+  <si>
+    <t>Referenced by TC-010.</t>
+  </si>
+  <si>
+    <t>TL-NFR-006</t>
+  </si>
+  <si>
+    <t>Sufficient evidence must be retained to reconstruct the mortgage-forbearance decision path from assessment through approval and execution.</t>
+  </si>
+  <si>
+    <t>Supports audit, compliance and quality-assurance review.</t>
+  </si>
+  <si>
+    <t>Audit history / decision reconstruction</t>
+  </si>
+  <si>
+    <t>Policy exception requires reason, evidence and authorised approval.</t>
+  </si>
+  <si>
+    <t>Policy exception cannot progress without authorised review and approval.</t>
+  </si>
+  <si>
+    <t>Direct exception-control scenario</t>
+  </si>
+  <si>
+    <t>Material case change after approval invalidates or supersedes prior approval.</t>
+  </si>
+  <si>
+    <t>Material change requires reassessment and new approval before execution.</t>
+  </si>
+  <si>
+    <t>Direct stale-approval scenario</t>
+  </si>
+  <si>
+    <t>Failed execution must not be treated as successful completion.</t>
+  </si>
+  <si>
+    <t>Failed execution is recorded and case remains incomplete.</t>
+  </si>
+  <si>
+    <t>Direct execution-failure scenario</t>
+  </si>
+  <si>
+    <t>Expired or previously used execution authorisation must not permit execution.</t>
+  </si>
+  <si>
+    <t>Reused or invalid authorisation is blocked and recorded.</t>
+  </si>
+  <si>
+    <t>Direct duplicate-authorisation scenario</t>
+  </si>
+  <si>
+    <t>Material actions must be timestamped and attributable to a user or system.</t>
+  </si>
+  <si>
+    <t>Audit history identifies actor/system, action and timestamp.</t>
+  </si>
+  <si>
+    <t>Auditability coverage</t>
+  </si>
+  <si>
+    <t>Sufficient evidence must be retained to reconstruct the decision path.</t>
+  </si>
+  <si>
+    <t>Reviewer can reconstruct evidence, rules, rationale, approval and execution history.</t>
+  </si>
+  <si>
+    <t>Decision-reconstruction coverage</t>
+  </si>
+  <si>
+    <t>TC-011</t>
+  </si>
+  <si>
+    <t>TL-FR-006, TL-RULE-003</t>
+  </si>
+  <si>
+    <t>Attempt to submit a proposed outcome without a recorded rationale</t>
+  </si>
+  <si>
+    <t>A mortgage-forbearance case has been assessed and a proposed outcome has been selected</t>
+  </si>
+  <si>
+    <t>1. Leave the decision rationale blank. 2. Attempt to submit the case for approval.</t>
+  </si>
+  <si>
+    <t>Submission is blocked because the proposed decision does not contain a recorded rationale, and the user is prompted to provide one.</t>
+  </si>
+  <si>
+    <t>TC-012</t>
+  </si>
+  <si>
+    <t>Review a submitted case and use each supported approval outcome</t>
+  </si>
+  <si>
+    <t>A complete case has been submitted to an authorised approver</t>
+  </si>
+  <si>
+    <t>1. Open the submitted case. 2. Confirm the Approve option is available. 3. Confirm the Reject option is available. 4. Confirm the Return for further information option is available. 5. Verify that rejecting or returning requires a reason or comment.</t>
+  </si>
+  <si>
+    <t>The authorised approver can approve, reject or return the case. Rejection and return actions require the relevant reason or comment to be recorded.</t>
+  </si>
+  <si>
+    <t>TC-013</t>
+  </si>
+  <si>
+    <t>TL-RULE-008, TL-FR-010</t>
+  </si>
+  <si>
+    <t>Change an approved decision and create a new controlled decision version</t>
+  </si>
+  <si>
+    <t>A mortgage-forbearance decision has already been approved and has a recorded decision version</t>
+  </si>
+  <si>
+    <t>1. Open the approved case. 2. Change a material element of the approved decision. 3. Save the change. 4. Review the decision history and version information.</t>
+  </si>
+  <si>
+    <t>The approved decision is not overwritten. A new controlled decision version is created, the previous version remains in the history, and the new version requires appropriate reassessment and approval before execution.</t>
+  </si>
+  <si>
+    <t>Column1</t>
   </si>
 </sst>
 </file>
@@ -313,14 +1245,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -331,6 +1282,110 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6E6DBA9D-3FB3-4466-9AF2-13EE2979FE0C}" name="Table1" displayName="Table1" ref="A1:H1048576" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:H1048576" xr:uid="{6E6DBA9D-3FB3-4466-9AF2-13EE2979FE0C}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{FC023ACA-E4A6-4BF7-87AB-1965C4179173}" name="Test Case ID"/>
+    <tableColumn id="2" xr3:uid="{C6D8FBC8-4675-49E0-A665-A09F9C08C528}" name="Requirement ID"/>
+    <tableColumn id="3" xr3:uid="{46BD1D82-9940-4615-997B-C740F8388849}" name="Scenario"/>
+    <tableColumn id="4" xr3:uid="{2170D162-087E-4546-AE0E-0F4CA761E4B1}" name="Preconditions"/>
+    <tableColumn id="5" xr3:uid="{80FA2419-AC7E-4FCD-A6EA-B3D01A071167}" name="Test Steps"/>
+    <tableColumn id="6" xr3:uid="{48330639-19D1-42B4-9385-4585ECC5DF7A}" name="Expected Result"/>
+    <tableColumn id="7" xr3:uid="{19C4182B-B291-4234-B7CB-88BCB7F64A19}" name="Actual Result"/>
+    <tableColumn id="8" xr3:uid="{FB72650E-965F-4CA5-B4D4-245D16BCE5FF}" name="Status"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{C17E521E-0B71-4EF0-B049-47F4EE7758A3}" name="Table6" displayName="Table6" ref="A1:H1048576" totalsRowShown="0">
+  <autoFilter ref="A1:H1048576" xr:uid="{C17E521E-0B71-4EF0-B049-47F4EE7758A3}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{FBB23155-6DD6-46B2-86C7-5FC9A7CF1CA8}" name="Requirement ID"/>
+    <tableColumn id="2" xr3:uid="{44218915-039A-4C5E-8DC2-87CCC9AA8922}" name="Requirement Description"/>
+    <tableColumn id="3" xr3:uid="{05F30139-310A-4DC0-8512-94F7CC35B27C}" name="Jira Story"/>
+    <tableColumn id="4" xr3:uid="{AD388908-6A65-4C72-8A89-0DBCE03CBF0D}" name="Acceptance Criteria"/>
+    <tableColumn id="5" xr3:uid="{73C76C27-4E9B-4797-ADBD-FE2E0D80FAC8}" name="Test Case ID"/>
+    <tableColumn id="6" xr3:uid="{A0E6DDEB-D697-4178-9DCC-56DD99690716}" name="Coverage Status"/>
+    <tableColumn id="7" xr3:uid="{FAFB3A70-8602-4C8D-A711-0AC385257422}" name="Comments"/>
+    <tableColumn id="8" xr3:uid="{A0767A45-E861-46CC-B89B-944A68E61E68}" name="Column1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{F245EB9A-3A1F-4D0D-9E41-77FE02A56812}" name="Table5" displayName="Table5" ref="A1:I1048576" totalsRowShown="0">
+  <autoFilter ref="A1:I1048576" xr:uid="{F245EB9A-3A1F-4D0D-9E41-77FE02A56812}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{5AB3C377-4CDE-4C79-8384-F728ABD201C0}" name="Requirement ID"/>
+    <tableColumn id="2" xr3:uid="{B254F3A7-901E-4BCE-B60A-C8300426D200}" name="Requirement Type"/>
+    <tableColumn id="3" xr3:uid="{5C0F4BB5-4A20-4B1D-B83E-25B9FAD0DFA5}" name="Requirement Description"/>
+    <tableColumn id="4" xr3:uid="{C6D13B21-66BD-41F4-817F-0AA953790E4A}" name="Source / Rationale"/>
+    <tableColumn id="5" xr3:uid="{8A98E3D2-5D04-4764-993F-49BBEED37CCC}" name="Priority"/>
+    <tableColumn id="6" xr3:uid="{6A54ED62-1FD0-4408-BFB9-779254FB66CC}" name="Status"/>
+    <tableColumn id="7" xr3:uid="{A7511E5B-0E76-436E-BE86-CBB6BAC1C16C}" name="Related Process Step"/>
+    <tableColumn id="8" xr3:uid="{E085AA21-3094-4B74-9515-01558087B477}" name="Related Rule ID"/>
+    <tableColumn id="9" xr3:uid="{BF0F12B1-E32D-4BC6-BADD-2068CAF0E8A4}" name="Comments"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{7FDD5C32-1AF3-4ACE-B625-839E4435209D}" name="Table7" displayName="Table7" ref="A1:I1048576" totalsRowShown="0">
+  <autoFilter ref="A1:I1048576" xr:uid="{7FDD5C32-1AF3-4ACE-B625-839E4435209D}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{2038363B-14B3-4470-9EBA-3F9A0661B47C}" name="Rule ID"/>
+    <tableColumn id="2" xr3:uid="{D569C22B-512D-499F-B173-31AE3198A001}" name="Rule Description"/>
+    <tableColumn id="3" xr3:uid="{03DF4F17-38C9-438A-B32B-8EDA37F65964}" name="Rule Type"/>
+    <tableColumn id="4" xr3:uid="{910E0E6F-8538-467C-8068-3EB3702CDE6A}" name="Trigger / Condition"/>
+    <tableColumn id="5" xr3:uid="{0F923038-74EA-45CA-BF32-D5522439AC80}" name="Expected Behaviour"/>
+    <tableColumn id="6" xr3:uid="{6A09F28E-CCBC-4D4C-A3F3-91FAB2B40616}" name="Exception Handling"/>
+    <tableColumn id="7" xr3:uid="{7B9EB2DC-7EE3-4754-A47E-9730B60A3A26}" name="Status"/>
+    <tableColumn id="8" xr3:uid="{01770764-0E18-4002-A865-842581B43928}" name="Related Requirement ID"/>
+    <tableColumn id="9" xr3:uid="{EB67BBA6-CB6E-4905-8D42-4E0F0B9B21D5}" name="Comments"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{1489E160-E589-47F0-9FF2-3FC9BCAF742D}" name="Table8" displayName="Table8" ref="A1:H1048576" totalsRowShown="0">
+  <autoFilter ref="A1:H1048576" xr:uid="{1489E160-E589-47F0-9FF2-3FC9BCAF742D}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{3EB878A8-EBCF-4350-95D7-86272239C36D}" name="Exception ID"/>
+    <tableColumn id="2" xr3:uid="{4F7D08D1-AC5A-408C-BD5A-92C305E686C1}" name="Exception Rule"/>
+    <tableColumn id="3" xr3:uid="{D8315EC9-3FAB-45E0-BDFA-113478340D08}" name="Trigger / Condition"/>
+    <tableColumn id="4" xr3:uid="{43C6B3BD-CECD-47EE-93F4-059BBCDE3200}" name="Expected Behaviour"/>
+    <tableColumn id="5" xr3:uid="{582E700C-5582-46DA-9FB2-AF4327920E7C}" name="Required Approval / Control"/>
+    <tableColumn id="6" xr3:uid="{DE086601-484F-4DC7-86D6-52CD15CE0E06}" name="Status"/>
+    <tableColumn id="7" xr3:uid="{36415B71-B0E4-4146-A395-3C8A8BA2106C}" name="Related Requirement / Rule"/>
+    <tableColumn id="8" xr3:uid="{DCC75D23-E4C6-450B-A79E-C062D20CF030}" name="Comments"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{DCFE65C6-A65C-4088-BC2D-9EC4C931B978}" name="Table10" displayName="Table10" ref="A1:H1048576" totalsRowShown="0">
+  <autoFilter ref="A1:H1048576" xr:uid="{DCFE65C6-A65C-4088-BC2D-9EC4C931B978}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{BDE47F78-9BAD-4BDC-9798-081503F2CCC1}" name="NFR ID"/>
+    <tableColumn id="2" xr3:uid="{FA37EE4F-15DD-4CAA-B42A-19B1DE5C85B9}" name="Category"/>
+    <tableColumn id="3" xr3:uid="{24D2C416-0693-4971-AC7F-0839FFC0894B}" name="Requirement Description"/>
+    <tableColumn id="4" xr3:uid="{219F7245-BF21-4D91-A748-355328A5E942}" name="Rationale"/>
+    <tableColumn id="5" xr3:uid="{B8E7B23D-7F2C-47D2-9086-3A8AFB13AC2A}" name="Priority"/>
+    <tableColumn id="6" xr3:uid="{905BE8BE-BB7C-4118-9D1C-E0CD7A28E75B}" name="Status"/>
+    <tableColumn id="7" xr3:uid="{DAF1F9FE-8DEB-439A-A6CC-71A75E37ADAF}" name="Related Process / Control"/>
+    <tableColumn id="8" xr3:uid="{19A5D4D0-7022-45BA-A82D-B10F61A349A1}" name="Comments"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -650,9 +1705,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4FFD6A5-3E80-46A6-BC2C-C73BA34AFEE9}">
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="1" max="1" width="13.6328125" customWidth="1"/>
     <col min="2" max="2" width="19.36328125" customWidth="1"/>
     <col min="3" max="3" width="39.26953125" customWidth="1"/>
     <col min="4" max="4" width="35.08984375" customWidth="1"/>
@@ -707,7 +1763,7 @@
         <v>13</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D2" t="s">
         <v>14</v>
@@ -727,42 +1783,42 @@
         <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>72</v>
       </c>
       <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" t="s">
         <v>21</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>22</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>23</v>
-      </c>
-      <c r="F3" t="s">
-        <v>24</v>
       </c>
       <c r="H3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="29" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" t="s">
         <v>25</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" t="s">
         <v>27</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>28</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>29</v>
-      </c>
-      <c r="F4" t="s">
-        <v>30</v>
       </c>
       <c r="H4" t="s">
         <v>17</v>
@@ -770,22 +1826,22 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
         <v>31</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>32</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>33</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>34</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>35</v>
-      </c>
-      <c r="F5" t="s">
-        <v>36</v>
       </c>
       <c r="H5" t="s">
         <v>17</v>
@@ -793,22 +1849,22 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" t="s">
         <v>37</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>38</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>39</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>40</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>41</v>
-      </c>
-      <c r="F6" t="s">
-        <v>42</v>
       </c>
       <c r="H6" t="s">
         <v>17</v>
@@ -816,22 +1872,22 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" t="s">
         <v>43</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>44</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>45</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>46</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>47</v>
-      </c>
-      <c r="F7" t="s">
-        <v>48</v>
       </c>
       <c r="H7" t="s">
         <v>17</v>
@@ -839,22 +1895,22 @@
     </row>
     <row r="8" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" t="s">
         <v>49</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" t="s">
         <v>51</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>52</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>53</v>
-      </c>
-      <c r="F8" t="s">
-        <v>54</v>
       </c>
       <c r="H8" t="s">
         <v>17</v>
@@ -862,22 +1918,22 @@
     </row>
     <row r="9" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" t="s">
         <v>55</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" t="s">
         <v>57</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>58</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>59</v>
-      </c>
-      <c r="F9" t="s">
-        <v>60</v>
       </c>
       <c r="H9" t="s">
         <v>17</v>
@@ -885,22 +1941,22 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" t="s">
         <v>61</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>62</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>63</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>64</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>65</v>
-      </c>
-      <c r="F10" t="s">
-        <v>66</v>
       </c>
       <c r="H10" t="s">
         <v>17</v>
@@ -908,30 +1964,1850 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" t="s">
         <v>67</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>68</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>69</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>70</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>71</v>
-      </c>
-      <c r="F11" t="s">
-        <v>72</v>
       </c>
       <c r="H11" t="s">
         <v>17</v>
       </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>364</v>
+      </c>
+      <c r="B12" t="s">
+        <v>365</v>
+      </c>
+      <c r="C12" t="s">
+        <v>366</v>
+      </c>
+      <c r="D12" t="s">
+        <v>367</v>
+      </c>
+      <c r="E12" t="s">
+        <v>368</v>
+      </c>
+      <c r="F12" t="s">
+        <v>369</v>
+      </c>
+      <c r="H12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>370</v>
+      </c>
+      <c r="B13" t="s">
+        <v>125</v>
+      </c>
+      <c r="C13" t="s">
+        <v>371</v>
+      </c>
+      <c r="D13" t="s">
+        <v>372</v>
+      </c>
+      <c r="E13" t="s">
+        <v>373</v>
+      </c>
+      <c r="F13" t="s">
+        <v>374</v>
+      </c>
+      <c r="H13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>375</v>
+      </c>
+      <c r="B14" t="s">
+        <v>376</v>
+      </c>
+      <c r="C14" t="s">
+        <v>377</v>
+      </c>
+      <c r="D14" t="s">
+        <v>378</v>
+      </c>
+      <c r="E14" t="s">
+        <v>379</v>
+      </c>
+      <c r="F14" t="s">
+        <v>380</v>
+      </c>
+      <c r="H14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A15" s="2"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A16" s="2"/>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="2"/>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" s="2"/>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" s="2"/>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" s="2"/>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" s="2"/>
+      <c r="B21" s="3"/>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" s="2"/>
+      <c r="B23" s="2"/>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" s="2"/>
+      <c r="B25" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B09CE922-E122-4EE6-B7F9-D904BA00C8E5}">
+  <dimension ref="A1:H33"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15.7265625" customWidth="1"/>
+    <col min="2" max="2" width="23.6328125" customWidth="1"/>
+    <col min="3" max="3" width="10.36328125" customWidth="1"/>
+    <col min="4" max="4" width="19.08984375" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="6" max="6" width="16.08984375" customWidth="1"/>
+    <col min="7" max="7" width="11.90625" customWidth="1"/>
+    <col min="8" max="8" width="10.36328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" t="s">
+        <v>76</v>
+      </c>
+      <c r="G1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C2" t="s">
+        <v>210</v>
+      </c>
+      <c r="D2" t="s">
+        <v>211</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>212</v>
+      </c>
+      <c r="G2" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" t="s">
+        <v>214</v>
+      </c>
+      <c r="C3" t="s">
+        <v>210</v>
+      </c>
+      <c r="D3" t="s">
+        <v>215</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
+        <v>212</v>
+      </c>
+      <c r="G3" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B4" t="s">
+        <v>216</v>
+      </c>
+      <c r="C4" t="s">
+        <v>217</v>
+      </c>
+      <c r="D4" t="s">
+        <v>218</v>
+      </c>
+      <c r="E4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" t="s">
+        <v>212</v>
+      </c>
+      <c r="G4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B5" t="s">
+        <v>220</v>
+      </c>
+      <c r="C5" t="s">
+        <v>221</v>
+      </c>
+      <c r="D5" t="s">
+        <v>222</v>
+      </c>
+      <c r="E5" t="s">
+        <v>48</v>
+      </c>
+      <c r="F5" t="s">
+        <v>223</v>
+      </c>
+      <c r="G5" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B6" t="s">
+        <v>225</v>
+      </c>
+      <c r="C6" t="s">
+        <v>221</v>
+      </c>
+      <c r="D6" t="s">
+        <v>226</v>
+      </c>
+      <c r="E6" t="s">
+        <v>66</v>
+      </c>
+      <c r="F6" t="s">
+        <v>223</v>
+      </c>
+      <c r="G6" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>111</v>
+      </c>
+      <c r="B7" t="s">
+        <v>228</v>
+      </c>
+      <c r="C7" t="s">
+        <v>221</v>
+      </c>
+      <c r="D7" t="s">
+        <v>229</v>
+      </c>
+      <c r="F7" t="s">
+        <v>230</v>
+      </c>
+      <c r="G7" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>116</v>
+      </c>
+      <c r="B8" t="s">
+        <v>232</v>
+      </c>
+      <c r="C8" t="s">
+        <v>233</v>
+      </c>
+      <c r="D8" t="s">
+        <v>234</v>
+      </c>
+      <c r="E8" t="s">
+        <v>235</v>
+      </c>
+      <c r="F8" t="s">
+        <v>223</v>
+      </c>
+      <c r="G8" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B9" t="s">
+        <v>237</v>
+      </c>
+      <c r="C9" t="s">
+        <v>238</v>
+      </c>
+      <c r="D9" t="s">
+        <v>239</v>
+      </c>
+      <c r="E9" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9" t="s">
+        <v>212</v>
+      </c>
+      <c r="G9" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>125</v>
+      </c>
+      <c r="B10" t="s">
+        <v>241</v>
+      </c>
+      <c r="C10" t="s">
+        <v>242</v>
+      </c>
+      <c r="D10" t="s">
+        <v>243</v>
+      </c>
+      <c r="F10" t="s">
+        <v>230</v>
+      </c>
+      <c r="G10" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>128</v>
+      </c>
+      <c r="B11" t="s">
+        <v>245</v>
+      </c>
+      <c r="C11" t="s">
+        <v>246</v>
+      </c>
+      <c r="D11" t="s">
+        <v>247</v>
+      </c>
+      <c r="E11" t="s">
+        <v>248</v>
+      </c>
+      <c r="F11" t="s">
+        <v>212</v>
+      </c>
+      <c r="G11" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>132</v>
+      </c>
+      <c r="B12" t="s">
+        <v>250</v>
+      </c>
+      <c r="C12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D12" t="s">
+        <v>252</v>
+      </c>
+      <c r="E12" t="s">
+        <v>248</v>
+      </c>
+      <c r="F12" t="s">
+        <v>212</v>
+      </c>
+      <c r="G12" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>138</v>
+      </c>
+      <c r="B13" t="s">
+        <v>254</v>
+      </c>
+      <c r="C13" t="s">
+        <v>251</v>
+      </c>
+      <c r="D13" t="s">
+        <v>255</v>
+      </c>
+      <c r="E13" t="s">
+        <v>256</v>
+      </c>
+      <c r="F13" t="s">
+        <v>212</v>
+      </c>
+      <c r="G13" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>143</v>
+      </c>
+      <c r="B14" t="s">
+        <v>258</v>
+      </c>
+      <c r="C14" t="s">
+        <v>259</v>
+      </c>
+      <c r="D14" t="s">
+        <v>260</v>
+      </c>
+      <c r="E14" t="s">
+        <v>66</v>
+      </c>
+      <c r="F14" t="s">
+        <v>212</v>
+      </c>
+      <c r="G14" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>148</v>
+      </c>
+      <c r="B15" t="s">
+        <v>262</v>
+      </c>
+      <c r="C15" t="s">
+        <v>259</v>
+      </c>
+      <c r="D15" t="s">
+        <v>263</v>
+      </c>
+      <c r="E15" t="s">
+        <v>66</v>
+      </c>
+      <c r="F15" t="s">
+        <v>212</v>
+      </c>
+      <c r="G15" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>98</v>
+      </c>
+      <c r="B17" t="s">
+        <v>265</v>
+      </c>
+      <c r="C17" t="s">
+        <v>266</v>
+      </c>
+      <c r="D17" t="s">
+        <v>267</v>
+      </c>
+      <c r="E17" t="s">
+        <v>18</v>
+      </c>
+      <c r="F17" t="s">
+        <v>212</v>
+      </c>
+      <c r="G17" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>107</v>
+      </c>
+      <c r="B18" t="s">
+        <v>269</v>
+      </c>
+      <c r="C18" t="s">
+        <v>270</v>
+      </c>
+      <c r="D18" t="s">
+        <v>271</v>
+      </c>
+      <c r="E18" t="s">
+        <v>272</v>
+      </c>
+      <c r="F18" t="s">
+        <v>223</v>
+      </c>
+      <c r="G18" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>115</v>
+      </c>
+      <c r="B19" t="s">
+        <v>274</v>
+      </c>
+      <c r="C19" t="s">
+        <v>275</v>
+      </c>
+      <c r="D19" t="s">
+        <v>276</v>
+      </c>
+      <c r="F19" t="s">
+        <v>230</v>
+      </c>
+      <c r="G19" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>120</v>
+      </c>
+      <c r="B20" t="s">
+        <v>278</v>
+      </c>
+      <c r="C20" t="s">
+        <v>238</v>
+      </c>
+      <c r="D20" t="s">
+        <v>279</v>
+      </c>
+      <c r="E20" t="s">
+        <v>235</v>
+      </c>
+      <c r="F20" t="s">
+        <v>223</v>
+      </c>
+      <c r="G20" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>124</v>
+      </c>
+      <c r="B21" t="s">
+        <v>281</v>
+      </c>
+      <c r="C21" t="s">
+        <v>238</v>
+      </c>
+      <c r="D21" t="s">
+        <v>282</v>
+      </c>
+      <c r="E21" t="s">
+        <v>24</v>
+      </c>
+      <c r="F21" t="s">
+        <v>212</v>
+      </c>
+      <c r="G21" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>131</v>
+      </c>
+      <c r="B22" t="s">
+        <v>284</v>
+      </c>
+      <c r="C22" t="s">
+        <v>285</v>
+      </c>
+      <c r="D22" t="s">
+        <v>286</v>
+      </c>
+      <c r="E22" t="s">
+        <v>287</v>
+      </c>
+      <c r="F22" t="s">
+        <v>212</v>
+      </c>
+      <c r="G22" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>187</v>
+      </c>
+      <c r="B23" t="s">
+        <v>288</v>
+      </c>
+      <c r="C23" t="s">
+        <v>289</v>
+      </c>
+      <c r="D23" t="s">
+        <v>290</v>
+      </c>
+      <c r="E23" t="s">
+        <v>42</v>
+      </c>
+      <c r="F23" t="s">
+        <v>212</v>
+      </c>
+      <c r="G23" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>193</v>
+      </c>
+      <c r="B24" t="s">
+        <v>292</v>
+      </c>
+      <c r="C24" t="s">
+        <v>285</v>
+      </c>
+      <c r="D24" t="s">
+        <v>293</v>
+      </c>
+      <c r="F24" t="s">
+        <v>230</v>
+      </c>
+      <c r="G24" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>142</v>
+      </c>
+      <c r="B25" t="s">
+        <v>295</v>
+      </c>
+      <c r="C25" t="s">
+        <v>296</v>
+      </c>
+      <c r="D25" t="s">
+        <v>297</v>
+      </c>
+      <c r="E25" t="s">
+        <v>256</v>
+      </c>
+      <c r="F25" t="s">
+        <v>212</v>
+      </c>
+      <c r="G25" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>147</v>
+      </c>
+      <c r="B26" t="s">
+        <v>299</v>
+      </c>
+      <c r="C26" t="s">
+        <v>300</v>
+      </c>
+      <c r="D26" t="s">
+        <v>301</v>
+      </c>
+      <c r="E26" t="s">
+        <v>66</v>
+      </c>
+      <c r="F26" t="s">
+        <v>212</v>
+      </c>
+      <c r="G26" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>307</v>
+      </c>
+      <c r="B28" t="s">
+        <v>346</v>
+      </c>
+      <c r="C28" t="s">
+        <v>238</v>
+      </c>
+      <c r="D28" t="s">
+        <v>347</v>
+      </c>
+      <c r="E28" t="s">
+        <v>48</v>
+      </c>
+      <c r="F28" t="s">
+        <v>212</v>
+      </c>
+      <c r="G28" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>314</v>
+      </c>
+      <c r="B29" t="s">
+        <v>349</v>
+      </c>
+      <c r="C29" t="s">
+        <v>289</v>
+      </c>
+      <c r="D29" t="s">
+        <v>350</v>
+      </c>
+      <c r="E29" t="s">
+        <v>42</v>
+      </c>
+      <c r="F29" t="s">
+        <v>212</v>
+      </c>
+      <c r="G29" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>321</v>
+      </c>
+      <c r="B30" t="s">
+        <v>352</v>
+      </c>
+      <c r="C30" t="s">
+        <v>285</v>
+      </c>
+      <c r="D30" t="s">
+        <v>353</v>
+      </c>
+      <c r="E30" t="s">
+        <v>60</v>
+      </c>
+      <c r="F30" t="s">
+        <v>212</v>
+      </c>
+      <c r="G30" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>55</v>
+      </c>
+      <c r="B31" t="s">
+        <v>355</v>
+      </c>
+      <c r="C31" t="s">
+        <v>285</v>
+      </c>
+      <c r="D31" t="s">
+        <v>356</v>
+      </c>
+      <c r="E31" t="s">
+        <v>54</v>
+      </c>
+      <c r="F31" t="s">
+        <v>212</v>
+      </c>
+      <c r="G31" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>337</v>
+      </c>
+      <c r="B32" t="s">
+        <v>358</v>
+      </c>
+      <c r="C32" t="s">
+        <v>300</v>
+      </c>
+      <c r="D32" t="s">
+        <v>359</v>
+      </c>
+      <c r="E32" t="s">
+        <v>66</v>
+      </c>
+      <c r="F32" t="s">
+        <v>212</v>
+      </c>
+      <c r="G32" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>342</v>
+      </c>
+      <c r="B33" t="s">
+        <v>361</v>
+      </c>
+      <c r="C33" t="s">
+        <v>300</v>
+      </c>
+      <c r="D33" t="s">
+        <v>362</v>
+      </c>
+      <c r="E33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F33" t="s">
+        <v>212</v>
+      </c>
+      <c r="G33" t="s">
+        <v>363</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4233A819-5076-48ED-8058-D5446539BE84}">
+  <dimension ref="A1:I15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15.7265625" customWidth="1"/>
+    <col min="2" max="2" width="17.7265625" customWidth="1"/>
+    <col min="3" max="3" width="23.6328125" customWidth="1"/>
+    <col min="4" max="4" width="18.1796875" customWidth="1"/>
+    <col min="5" max="5" width="8.90625" customWidth="1"/>
+    <col min="7" max="7" width="20.1796875" customWidth="1"/>
+    <col min="8" max="8" width="15.453125" customWidth="1"/>
+    <col min="9" max="9" width="11.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" t="s">
+        <v>80</v>
+      </c>
+      <c r="H1" t="s">
+        <v>81</v>
+      </c>
+      <c r="I1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D2" t="s">
+        <v>91</v>
+      </c>
+      <c r="E2" t="s">
+        <v>92</v>
+      </c>
+      <c r="F2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C3" t="s">
+        <v>96</v>
+      </c>
+      <c r="D3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E3" t="s">
+        <v>92</v>
+      </c>
+      <c r="F3" t="s">
+        <v>93</v>
+      </c>
+      <c r="G3" t="s">
+        <v>94</v>
+      </c>
+      <c r="H3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E4" t="s">
+        <v>92</v>
+      </c>
+      <c r="F4" t="s">
+        <v>93</v>
+      </c>
+      <c r="G4" t="s">
+        <v>102</v>
+      </c>
+      <c r="H4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D5" t="s">
+        <v>105</v>
+      </c>
+      <c r="E5" t="s">
+        <v>92</v>
+      </c>
+      <c r="F5" t="s">
+        <v>93</v>
+      </c>
+      <c r="G5" t="s">
+        <v>106</v>
+      </c>
+      <c r="H5" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B6" t="s">
+        <v>89</v>
+      </c>
+      <c r="C6" t="s">
+        <v>109</v>
+      </c>
+      <c r="D6" t="s">
+        <v>110</v>
+      </c>
+      <c r="E6" t="s">
+        <v>92</v>
+      </c>
+      <c r="F6" t="s">
+        <v>93</v>
+      </c>
+      <c r="G6" t="s">
+        <v>106</v>
+      </c>
+      <c r="H6" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>111</v>
+      </c>
+      <c r="B7" t="s">
+        <v>89</v>
+      </c>
+      <c r="C7" t="s">
+        <v>112</v>
+      </c>
+      <c r="D7" t="s">
+        <v>113</v>
+      </c>
+      <c r="E7" t="s">
+        <v>92</v>
+      </c>
+      <c r="F7" t="s">
+        <v>93</v>
+      </c>
+      <c r="G7" t="s">
+        <v>114</v>
+      </c>
+      <c r="H7" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>116</v>
+      </c>
+      <c r="B8" t="s">
+        <v>89</v>
+      </c>
+      <c r="C8" t="s">
+        <v>117</v>
+      </c>
+      <c r="D8" t="s">
+        <v>118</v>
+      </c>
+      <c r="E8" t="s">
+        <v>92</v>
+      </c>
+      <c r="F8" t="s">
+        <v>93</v>
+      </c>
+      <c r="G8" t="s">
+        <v>119</v>
+      </c>
+      <c r="H8" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C9" t="s">
+        <v>122</v>
+      </c>
+      <c r="D9" t="s">
+        <v>123</v>
+      </c>
+      <c r="E9" t="s">
+        <v>92</v>
+      </c>
+      <c r="F9" t="s">
+        <v>93</v>
+      </c>
+      <c r="G9" t="s">
+        <v>119</v>
+      </c>
+      <c r="H9" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>125</v>
+      </c>
+      <c r="B10" t="s">
+        <v>89</v>
+      </c>
+      <c r="C10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D10" t="s">
+        <v>127</v>
+      </c>
+      <c r="E10" t="s">
+        <v>92</v>
+      </c>
+      <c r="F10" t="s">
+        <v>93</v>
+      </c>
+      <c r="G10" t="s">
+        <v>119</v>
+      </c>
+      <c r="H10" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>128</v>
+      </c>
+      <c r="B11" t="s">
+        <v>89</v>
+      </c>
+      <c r="C11" t="s">
+        <v>129</v>
+      </c>
+      <c r="D11" t="s">
+        <v>130</v>
+      </c>
+      <c r="E11" t="s">
+        <v>92</v>
+      </c>
+      <c r="F11" t="s">
+        <v>93</v>
+      </c>
+      <c r="G11" t="s">
+        <v>119</v>
+      </c>
+      <c r="H11" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>132</v>
+      </c>
+      <c r="B12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C12" t="s">
+        <v>133</v>
+      </c>
+      <c r="D12" t="s">
+        <v>134</v>
+      </c>
+      <c r="E12" t="s">
+        <v>135</v>
+      </c>
+      <c r="F12" t="s">
+        <v>93</v>
+      </c>
+      <c r="G12" t="s">
+        <v>136</v>
+      </c>
+      <c r="H12" t="s">
+        <v>131</v>
+      </c>
+      <c r="I12" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>138</v>
+      </c>
+      <c r="B13" t="s">
+        <v>89</v>
+      </c>
+      <c r="C13" t="s">
+        <v>139</v>
+      </c>
+      <c r="D13" t="s">
+        <v>140</v>
+      </c>
+      <c r="E13" t="s">
+        <v>92</v>
+      </c>
+      <c r="F13" t="s">
+        <v>93</v>
+      </c>
+      <c r="G13" t="s">
+        <v>141</v>
+      </c>
+      <c r="H13" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>143</v>
+      </c>
+      <c r="B14" t="s">
+        <v>89</v>
+      </c>
+      <c r="C14" t="s">
+        <v>144</v>
+      </c>
+      <c r="D14" t="s">
+        <v>145</v>
+      </c>
+      <c r="E14" t="s">
+        <v>92</v>
+      </c>
+      <c r="F14" t="s">
+        <v>93</v>
+      </c>
+      <c r="G14" t="s">
+        <v>146</v>
+      </c>
+      <c r="H14" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>148</v>
+      </c>
+      <c r="B15" t="s">
+        <v>89</v>
+      </c>
+      <c r="C15" t="s">
+        <v>149</v>
+      </c>
+      <c r="D15" t="s">
+        <v>150</v>
+      </c>
+      <c r="E15" t="s">
+        <v>92</v>
+      </c>
+      <c r="F15" t="s">
+        <v>93</v>
+      </c>
+      <c r="G15" t="s">
+        <v>146</v>
+      </c>
+      <c r="H15" t="s">
+        <v>147</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AD45A1F-46BF-4C09-A856-35CFFCA501DE}">
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.6328125" customWidth="1"/>
+    <col min="3" max="3" width="10.81640625" customWidth="1"/>
+    <col min="4" max="4" width="18.26953125" customWidth="1"/>
+    <col min="5" max="5" width="19.08984375" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
+    <col min="8" max="8" width="22.36328125" customWidth="1"/>
+    <col min="9" max="9" width="11.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" t="s">
+        <v>86</v>
+      </c>
+      <c r="F1" t="s">
+        <v>151</v>
+      </c>
+      <c r="G1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" t="s">
+        <v>87</v>
+      </c>
+      <c r="I1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E2" t="s">
+        <v>155</v>
+      </c>
+      <c r="F2" t="s">
+        <v>156</v>
+      </c>
+      <c r="G2" t="s">
+        <v>93</v>
+      </c>
+      <c r="H2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B3" t="s">
+        <v>158</v>
+      </c>
+      <c r="C3" t="s">
+        <v>159</v>
+      </c>
+      <c r="D3" t="s">
+        <v>160</v>
+      </c>
+      <c r="E3" t="s">
+        <v>161</v>
+      </c>
+      <c r="F3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G3" t="s">
+        <v>93</v>
+      </c>
+      <c r="H3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C4" t="s">
+        <v>165</v>
+      </c>
+      <c r="D4" t="s">
+        <v>166</v>
+      </c>
+      <c r="E4" t="s">
+        <v>167</v>
+      </c>
+      <c r="F4" t="s">
+        <v>168</v>
+      </c>
+      <c r="G4" t="s">
+        <v>93</v>
+      </c>
+      <c r="H4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>120</v>
+      </c>
+      <c r="B5" t="s">
+        <v>169</v>
+      </c>
+      <c r="C5" t="s">
+        <v>170</v>
+      </c>
+      <c r="D5" t="s">
+        <v>171</v>
+      </c>
+      <c r="E5" t="s">
+        <v>172</v>
+      </c>
+      <c r="F5" t="s">
+        <v>173</v>
+      </c>
+      <c r="G5" t="s">
+        <v>93</v>
+      </c>
+      <c r="H5" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>124</v>
+      </c>
+      <c r="B6" t="s">
+        <v>175</v>
+      </c>
+      <c r="C6" t="s">
+        <v>176</v>
+      </c>
+      <c r="D6" t="s">
+        <v>177</v>
+      </c>
+      <c r="E6" t="s">
+        <v>178</v>
+      </c>
+      <c r="F6" t="s">
+        <v>179</v>
+      </c>
+      <c r="G6" t="s">
+        <v>93</v>
+      </c>
+      <c r="H6" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>131</v>
+      </c>
+      <c r="B7" t="s">
+        <v>180</v>
+      </c>
+      <c r="C7" t="s">
+        <v>181</v>
+      </c>
+      <c r="D7" t="s">
+        <v>182</v>
+      </c>
+      <c r="E7" t="s">
+        <v>183</v>
+      </c>
+      <c r="F7" t="s">
+        <v>184</v>
+      </c>
+      <c r="G7" t="s">
+        <v>93</v>
+      </c>
+      <c r="H7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I7" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>187</v>
+      </c>
+      <c r="B8" t="s">
+        <v>188</v>
+      </c>
+      <c r="C8" t="s">
+        <v>189</v>
+      </c>
+      <c r="D8" t="s">
+        <v>190</v>
+      </c>
+      <c r="E8" t="s">
+        <v>191</v>
+      </c>
+      <c r="F8" t="s">
+        <v>192</v>
+      </c>
+      <c r="G8" t="s">
+        <v>93</v>
+      </c>
+      <c r="H8" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>193</v>
+      </c>
+      <c r="B9" t="s">
+        <v>194</v>
+      </c>
+      <c r="C9" t="s">
+        <v>189</v>
+      </c>
+      <c r="D9" t="s">
+        <v>195</v>
+      </c>
+      <c r="E9" t="s">
+        <v>196</v>
+      </c>
+      <c r="F9" t="s">
+        <v>197</v>
+      </c>
+      <c r="G9" t="s">
+        <v>93</v>
+      </c>
+      <c r="H9" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>142</v>
+      </c>
+      <c r="B10" t="s">
+        <v>198</v>
+      </c>
+      <c r="C10" t="s">
+        <v>199</v>
+      </c>
+      <c r="D10" t="s">
+        <v>200</v>
+      </c>
+      <c r="E10" t="s">
+        <v>201</v>
+      </c>
+      <c r="F10" t="s">
+        <v>202</v>
+      </c>
+      <c r="G10" t="s">
+        <v>93</v>
+      </c>
+      <c r="H10" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>147</v>
+      </c>
+      <c r="B11" t="s">
+        <v>203</v>
+      </c>
+      <c r="C11" t="s">
+        <v>204</v>
+      </c>
+      <c r="D11" t="s">
+        <v>205</v>
+      </c>
+      <c r="E11" t="s">
+        <v>206</v>
+      </c>
+      <c r="F11" t="s">
+        <v>207</v>
+      </c>
+      <c r="G11" t="s">
+        <v>93</v>
+      </c>
+      <c r="H11" t="s">
+        <v>208</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84A7C8F9-EDF9-4E39-B2A2-C3A84585CD27}">
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.08984375" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="18.26953125" customWidth="1"/>
+    <col min="4" max="4" width="19.08984375" customWidth="1"/>
+    <col min="5" max="5" width="25.90625" customWidth="1"/>
+    <col min="7" max="7" width="25.36328125" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>303</v>
+      </c>
+      <c r="B1" t="s">
+        <v>304</v>
+      </c>
+      <c r="C1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E1" t="s">
+        <v>305</v>
+      </c>
+      <c r="F1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" t="s">
+        <v>306</v>
+      </c>
+      <c r="H1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>307</v>
+      </c>
+      <c r="B2" t="s">
+        <v>308</v>
+      </c>
+      <c r="C2" t="s">
+        <v>309</v>
+      </c>
+      <c r="D2" t="s">
+        <v>310</v>
+      </c>
+      <c r="E2" t="s">
+        <v>311</v>
+      </c>
+      <c r="F2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G2" t="s">
+        <v>312</v>
+      </c>
+      <c r="H2" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>314</v>
+      </c>
+      <c r="B3" t="s">
+        <v>315</v>
+      </c>
+      <c r="C3" t="s">
+        <v>316</v>
+      </c>
+      <c r="D3" t="s">
+        <v>317</v>
+      </c>
+      <c r="E3" t="s">
+        <v>318</v>
+      </c>
+      <c r="F3" t="s">
+        <v>93</v>
+      </c>
+      <c r="G3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H3" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>321</v>
+      </c>
+      <c r="B4" t="s">
+        <v>322</v>
+      </c>
+      <c r="C4" t="s">
+        <v>323</v>
+      </c>
+      <c r="D4" t="s">
+        <v>324</v>
+      </c>
+      <c r="E4" t="s">
+        <v>325</v>
+      </c>
+      <c r="F4" t="s">
+        <v>93</v>
+      </c>
+      <c r="G4" t="s">
+        <v>326</v>
+      </c>
+      <c r="H4" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" t="s">
+        <v>328</v>
+      </c>
+      <c r="C5" t="s">
+        <v>329</v>
+      </c>
+      <c r="D5" t="s">
+        <v>330</v>
+      </c>
+      <c r="E5" t="s">
+        <v>331</v>
+      </c>
+      <c r="F5" t="s">
+        <v>93</v>
+      </c>
+      <c r="G5" t="s">
+        <v>132</v>
+      </c>
+      <c r="H5" t="s">
+        <v>332</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BC566F7-FFD1-4E99-8595-C7DE233A0F00}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="10.08984375" customWidth="1"/>
+    <col min="3" max="3" width="23.6328125" customWidth="1"/>
+    <col min="4" max="4" width="10.90625" customWidth="1"/>
+    <col min="5" max="5" width="8.90625" customWidth="1"/>
+    <col min="7" max="7" width="23.90625" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>333</v>
+      </c>
+      <c r="B1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D1" t="s">
+        <v>335</v>
+      </c>
+      <c r="E1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" t="s">
+        <v>336</v>
+      </c>
+      <c r="H1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>337</v>
+      </c>
+      <c r="B2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C2" t="s">
+        <v>339</v>
+      </c>
+      <c r="D2" t="s">
+        <v>340</v>
+      </c>
+      <c r="E2" t="s">
+        <v>92</v>
+      </c>
+      <c r="F2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G2" t="s">
+        <v>146</v>
+      </c>
+      <c r="H2" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>342</v>
+      </c>
+      <c r="B3" t="s">
+        <v>338</v>
+      </c>
+      <c r="C3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D3" t="s">
+        <v>344</v>
+      </c>
+      <c r="E3" t="s">
+        <v>92</v>
+      </c>
+      <c r="F3" t="s">
+        <v>93</v>
+      </c>
+      <c r="G3" t="s">
+        <v>345</v>
+      </c>
+      <c r="H3" t="s">
+        <v>341</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>